<commit_message>
Separar administración de reglas en programa externo con interfaz propia
</commit_message>
<xml_diff>
--- a/qgis_control_calidad/resources/plantillas/plantilla_reglas.xlsx
+++ b/qgis_control_calidad/resources/plantillas/plantilla_reglas.xlsx
@@ -3016,7 +3016,7 @@
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Elija el destino en Administrar reglas. El archivo no contiene credenciales ni decide el esquema de destino.</t>
+          <t>Elija el destino en el programa externo Administrador de reglas. El archivo no contiene credenciales ni decide el esquema de destino.</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3037,7 @@
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Revise la vista previa y pulse Incorporar reglas nuevas. Una falla revierte toda la operación.</t>
+          <t>Revise la vista previa y pulse Cargar reglas nuevas. Una falla revierte toda la operación.</t>
         </is>
       </c>
     </row>

</xml_diff>